<commit_message>
update data package at: 2026-09-25T20:00:55
</commit_message>
<xml_diff>
--- a/data/BASE_DETALHAMENTO_OBRAS.xlsx
+++ b/data/BASE_DETALHAMENTO_OBRAS.xlsx
@@ -930,10 +930,10 @@
         </is>
       </c>
       <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
         <v>60000</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0</v>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
@@ -1004,10 +1004,10 @@
         </is>
       </c>
       <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
         <v>197857</v>
-      </c>
-      <c r="R8" t="n">
-        <v>0</v>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
@@ -1078,10 +1078,10 @@
         </is>
       </c>
       <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
         <v>1929103</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0</v>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
@@ -1152,10 +1152,10 @@
         </is>
       </c>
       <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
         <v>1929103</v>
-      </c>
-      <c r="R10" t="n">
-        <v>0</v>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr"/>
@@ -1226,10 +1226,10 @@
         </is>
       </c>
       <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
         <v>41022</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0</v>
       </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
@@ -1300,10 +1300,10 @@
         </is>
       </c>
       <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" t="n">
         <v>100000</v>
-      </c>
-      <c r="R12" t="n">
-        <v>0</v>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr"/>
@@ -5380,10 +5380,10 @@
         </is>
       </c>
       <c r="Q72" t="n">
-        <v>280106</v>
+        <v>0</v>
       </c>
       <c r="R72" t="n">
-        <v>519640</v>
+        <v>799746</v>
       </c>
       <c r="S72" t="inlineStr"/>
       <c r="T72" t="inlineStr"/>
@@ -5448,10 +5448,10 @@
         </is>
       </c>
       <c r="Q73" t="n">
-        <v>894720</v>
+        <v>0</v>
       </c>
       <c r="R73" t="n">
-        <v>4087644</v>
+        <v>4982364</v>
       </c>
       <c r="S73" t="inlineStr"/>
       <c r="T73" t="inlineStr"/>
@@ -5516,10 +5516,10 @@
         </is>
       </c>
       <c r="Q74" t="n">
-        <v>8264640</v>
+        <v>0</v>
       </c>
       <c r="R74" t="n">
-        <v>19153735</v>
+        <v>27418375</v>
       </c>
       <c r="S74" t="inlineStr"/>
       <c r="T74" t="inlineStr"/>
@@ -5584,10 +5584,10 @@
         </is>
       </c>
       <c r="Q75" t="n">
-        <v>3155040</v>
+        <v>0</v>
       </c>
       <c r="R75" t="n">
-        <v>23943007</v>
+        <v>27098047</v>
       </c>
       <c r="S75" t="inlineStr"/>
       <c r="T75" t="inlineStr"/>
@@ -5652,10 +5652,10 @@
         </is>
       </c>
       <c r="Q76" t="n">
-        <v>4840800</v>
+        <v>0</v>
       </c>
       <c r="R76" t="n">
-        <v>26593690</v>
+        <v>31434490</v>
       </c>
       <c r="S76" t="inlineStr"/>
       <c r="T76" t="inlineStr"/>
@@ -5720,10 +5720,10 @@
         </is>
       </c>
       <c r="Q77" t="n">
-        <v>613500</v>
+        <v>0</v>
       </c>
       <c r="R77" t="n">
-        <v>2870210</v>
+        <v>3483710</v>
       </c>
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="inlineStr"/>
@@ -5788,10 +5788,10 @@
         </is>
       </c>
       <c r="Q78" t="n">
-        <v>5963400</v>
+        <v>0</v>
       </c>
       <c r="R78" t="n">
-        <v>23280000</v>
+        <v>29243400</v>
       </c>
       <c r="S78" t="inlineStr"/>
       <c r="T78" t="inlineStr"/>
@@ -5856,10 +5856,10 @@
         </is>
       </c>
       <c r="Q79" t="n">
-        <v>3620820</v>
+        <v>0</v>
       </c>
       <c r="R79" t="n">
-        <v>19100000</v>
+        <v>22720820</v>
       </c>
       <c r="S79" t="inlineStr"/>
       <c r="T79" t="inlineStr"/>
@@ -5990,10 +5990,10 @@
         </is>
       </c>
       <c r="Q81" t="n">
-        <v>1839798</v>
+        <v>0</v>
       </c>
       <c r="R81" t="n">
-        <v>3269655</v>
+        <v>5109453</v>
       </c>
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="inlineStr"/>
@@ -6058,10 +6058,10 @@
         </is>
       </c>
       <c r="Q82" t="n">
+        <v>0</v>
+      </c>
+      <c r="R82" t="n">
         <v>222899</v>
-      </c>
-      <c r="R82" t="n">
-        <v>0</v>
       </c>
       <c r="S82" t="inlineStr"/>
       <c r="T82" t="inlineStr"/>
@@ -7206,10 +7206,10 @@
         </is>
       </c>
       <c r="Q99" t="n">
+        <v>0</v>
+      </c>
+      <c r="R99" t="n">
         <v>299895</v>
-      </c>
-      <c r="R99" t="n">
-        <v>0</v>
       </c>
       <c r="S99" t="inlineStr"/>
       <c r="T99" t="inlineStr"/>
@@ -7274,10 +7274,10 @@
         </is>
       </c>
       <c r="Q100" t="n">
+        <v>0</v>
+      </c>
+      <c r="R100" t="n">
         <v>4565604</v>
-      </c>
-      <c r="R100" t="n">
-        <v>0</v>
       </c>
       <c r="S100" t="inlineStr"/>
       <c r="T100" t="inlineStr"/>
@@ -7342,10 +7342,10 @@
         </is>
       </c>
       <c r="Q101" t="n">
-        <v>6286532</v>
+        <v>0</v>
       </c>
       <c r="R101" t="n">
-        <v>2728583</v>
+        <v>9015115</v>
       </c>
       <c r="S101" t="inlineStr"/>
       <c r="T101" t="inlineStr"/>
@@ -7410,10 +7410,10 @@
         </is>
       </c>
       <c r="Q102" t="n">
+        <v>0</v>
+      </c>
+      <c r="R102" t="n">
         <v>193263</v>
-      </c>
-      <c r="R102" t="n">
-        <v>0</v>
       </c>
       <c r="S102" t="inlineStr"/>
       <c r="T102" t="inlineStr"/>
@@ -7608,10 +7608,10 @@
         </is>
       </c>
       <c r="Q105" t="n">
-        <v>904245</v>
+        <v>0</v>
       </c>
       <c r="R105" t="n">
-        <v>44308050</v>
+        <v>45212295</v>
       </c>
       <c r="S105" t="inlineStr"/>
       <c r="T105" t="inlineStr"/>
@@ -7674,10 +7674,10 @@
         </is>
       </c>
       <c r="Q106" t="n">
+        <v>0</v>
+      </c>
+      <c r="R106" t="n">
         <v>6999284</v>
-      </c>
-      <c r="R106" t="n">
-        <v>0</v>
       </c>
       <c r="S106" t="inlineStr"/>
       <c r="T106" t="inlineStr"/>
@@ -7740,10 +7740,10 @@
         </is>
       </c>
       <c r="Q107" t="n">
+        <v>0</v>
+      </c>
+      <c r="R107" t="n">
         <v>651694</v>
-      </c>
-      <c r="R107" t="n">
-        <v>0</v>
       </c>
       <c r="S107" t="inlineStr"/>
       <c r="T107" t="inlineStr"/>
@@ -7806,10 +7806,10 @@
         </is>
       </c>
       <c r="Q108" t="n">
+        <v>0</v>
+      </c>
+      <c r="R108" t="n">
         <v>651694</v>
-      </c>
-      <c r="R108" t="n">
-        <v>0</v>
       </c>
       <c r="S108" t="inlineStr"/>
       <c r="T108" t="inlineStr"/>
@@ -7872,10 +7872,10 @@
         </is>
       </c>
       <c r="Q109" t="n">
+        <v>0</v>
+      </c>
+      <c r="R109" t="n">
         <v>1472757</v>
-      </c>
-      <c r="R109" t="n">
-        <v>0</v>
       </c>
       <c r="S109" t="inlineStr"/>
       <c r="T109" t="inlineStr"/>
@@ -7938,10 +7938,10 @@
         </is>
       </c>
       <c r="Q110" t="n">
+        <v>0</v>
+      </c>
+      <c r="R110" t="n">
         <v>651694</v>
-      </c>
-      <c r="R110" t="n">
-        <v>0</v>
       </c>
       <c r="S110" t="inlineStr"/>
       <c r="T110" t="inlineStr"/>
@@ -8004,10 +8004,10 @@
         </is>
       </c>
       <c r="Q111" t="n">
+        <v>0</v>
+      </c>
+      <c r="R111" t="n">
         <v>18572878</v>
-      </c>
-      <c r="R111" t="n">
-        <v>0</v>
       </c>
       <c r="S111" t="inlineStr"/>
       <c r="T111" t="inlineStr"/>
@@ -8604,10 +8604,10 @@
         </is>
       </c>
       <c r="Q120" t="n">
-        <v>150000</v>
+        <v>0</v>
       </c>
       <c r="R120" t="n">
-        <v>19850000</v>
+        <v>20000000</v>
       </c>
       <c r="S120" t="inlineStr"/>
       <c r="T120" t="inlineStr"/>
@@ -8946,10 +8946,10 @@
         </is>
       </c>
       <c r="Q125" t="n">
+        <v>0</v>
+      </c>
+      <c r="R125" t="n">
         <v>350000</v>
-      </c>
-      <c r="R125" t="n">
-        <v>0</v>
       </c>
       <c r="S125" t="inlineStr"/>
       <c r="T125" t="inlineStr"/>
@@ -9018,10 +9018,10 @@
         </is>
       </c>
       <c r="Q126" t="n">
+        <v>0</v>
+      </c>
+      <c r="R126" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R126" t="n">
-        <v>0</v>
       </c>
       <c r="S126" t="inlineStr"/>
       <c r="T126" t="inlineStr"/>
@@ -9814,10 +9814,10 @@
         </is>
       </c>
       <c r="Q138" t="n">
+        <v>0</v>
+      </c>
+      <c r="R138" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R138" t="n">
-        <v>0</v>
       </c>
       <c r="S138" t="inlineStr"/>
       <c r="T138" t="inlineStr"/>
@@ -9880,10 +9880,10 @@
         </is>
       </c>
       <c r="Q139" t="n">
+        <v>0</v>
+      </c>
+      <c r="R139" t="n">
         <v>143000</v>
-      </c>
-      <c r="R139" t="n">
-        <v>0</v>
       </c>
       <c r="S139" t="inlineStr"/>
       <c r="T139" t="inlineStr"/>
@@ -9946,10 +9946,10 @@
         </is>
       </c>
       <c r="Q140" t="n">
+        <v>0</v>
+      </c>
+      <c r="R140" t="n">
         <v>5876140</v>
-      </c>
-      <c r="R140" t="n">
-        <v>0</v>
       </c>
       <c r="S140" t="inlineStr"/>
       <c r="T140" t="inlineStr"/>
@@ -10012,10 +10012,10 @@
         </is>
       </c>
       <c r="Q141" t="n">
+        <v>0</v>
+      </c>
+      <c r="R141" t="n">
         <v>1132500</v>
-      </c>
-      <c r="R141" t="n">
-        <v>0</v>
       </c>
       <c r="S141" t="inlineStr"/>
       <c r="T141" t="inlineStr"/>
@@ -10078,10 +10078,10 @@
         </is>
       </c>
       <c r="Q142" t="n">
+        <v>0</v>
+      </c>
+      <c r="R142" t="n">
         <v>34710000</v>
-      </c>
-      <c r="R142" t="n">
-        <v>0</v>
       </c>
       <c r="S142" t="inlineStr"/>
       <c r="T142" t="inlineStr"/>
@@ -10144,10 +10144,10 @@
         </is>
       </c>
       <c r="Q143" t="n">
+        <v>0</v>
+      </c>
+      <c r="R143" t="n">
         <v>59000000</v>
-      </c>
-      <c r="R143" t="n">
-        <v>0</v>
       </c>
       <c r="S143" t="inlineStr"/>
       <c r="T143" t="inlineStr"/>
@@ -10210,10 +10210,10 @@
         </is>
       </c>
       <c r="Q144" t="n">
+        <v>0</v>
+      </c>
+      <c r="R144" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R144" t="n">
-        <v>0</v>
       </c>
       <c r="S144" t="inlineStr"/>
       <c r="T144" t="inlineStr"/>
@@ -10276,10 +10276,10 @@
         </is>
       </c>
       <c r="Q145" t="n">
+        <v>0</v>
+      </c>
+      <c r="R145" t="n">
         <v>200000</v>
-      </c>
-      <c r="R145" t="n">
-        <v>0</v>
       </c>
       <c r="S145" t="inlineStr"/>
       <c r="T145" t="inlineStr"/>
@@ -10342,10 +10342,10 @@
         </is>
       </c>
       <c r="Q146" t="n">
+        <v>0</v>
+      </c>
+      <c r="R146" t="n">
         <v>30980000</v>
-      </c>
-      <c r="R146" t="n">
-        <v>0</v>
       </c>
       <c r="S146" t="inlineStr"/>
       <c r="T146" t="inlineStr"/>
@@ -10408,10 +10408,10 @@
         </is>
       </c>
       <c r="Q147" t="n">
+        <v>0</v>
+      </c>
+      <c r="R147" t="n">
         <v>25655000</v>
-      </c>
-      <c r="R147" t="n">
-        <v>0</v>
       </c>
       <c r="S147" t="inlineStr"/>
       <c r="T147" t="inlineStr"/>
@@ -10474,10 +10474,10 @@
         </is>
       </c>
       <c r="Q148" t="n">
+        <v>0</v>
+      </c>
+      <c r="R148" t="n">
         <v>66560000</v>
-      </c>
-      <c r="R148" t="n">
-        <v>0</v>
       </c>
       <c r="S148" t="inlineStr"/>
       <c r="T148" t="inlineStr"/>
@@ -10540,10 +10540,10 @@
         </is>
       </c>
       <c r="Q149" t="n">
+        <v>0</v>
+      </c>
+      <c r="R149" t="n">
         <v>25464500</v>
-      </c>
-      <c r="R149" t="n">
-        <v>0</v>
       </c>
       <c r="S149" t="inlineStr"/>
       <c r="T149" t="inlineStr"/>
@@ -10606,10 +10606,10 @@
         </is>
       </c>
       <c r="Q150" t="n">
+        <v>0</v>
+      </c>
+      <c r="R150" t="n">
         <v>1202905</v>
-      </c>
-      <c r="R150" t="n">
-        <v>0</v>
       </c>
       <c r="S150" t="inlineStr"/>
       <c r="T150" t="inlineStr"/>
@@ -10672,10 +10672,10 @@
         </is>
       </c>
       <c r="Q151" t="n">
+        <v>0</v>
+      </c>
+      <c r="R151" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R151" t="n">
-        <v>0</v>
       </c>
       <c r="S151" t="inlineStr"/>
       <c r="T151" t="inlineStr"/>
@@ -10738,10 +10738,10 @@
         </is>
       </c>
       <c r="Q152" t="n">
+        <v>0</v>
+      </c>
+      <c r="R152" t="n">
         <v>14920000</v>
-      </c>
-      <c r="R152" t="n">
-        <v>0</v>
       </c>
       <c r="S152" t="inlineStr"/>
       <c r="T152" t="inlineStr"/>
@@ -10804,10 +10804,10 @@
         </is>
       </c>
       <c r="Q153" t="n">
+        <v>0</v>
+      </c>
+      <c r="R153" t="n">
         <v>8798400</v>
-      </c>
-      <c r="R153" t="n">
-        <v>0</v>
       </c>
       <c r="S153" t="inlineStr"/>
       <c r="T153" t="inlineStr"/>
@@ -10870,10 +10870,10 @@
         </is>
       </c>
       <c r="Q154" t="n">
+        <v>0</v>
+      </c>
+      <c r="R154" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R154" t="n">
-        <v>0</v>
       </c>
       <c r="S154" t="inlineStr"/>
       <c r="T154" t="inlineStr"/>
@@ -10936,10 +10936,10 @@
         </is>
       </c>
       <c r="Q155" t="n">
+        <v>0</v>
+      </c>
+      <c r="R155" t="n">
         <v>1203643</v>
-      </c>
-      <c r="R155" t="n">
-        <v>0</v>
       </c>
       <c r="S155" t="inlineStr"/>
       <c r="T155" t="inlineStr"/>
@@ -11002,10 +11002,10 @@
         </is>
       </c>
       <c r="Q156" t="n">
+        <v>0</v>
+      </c>
+      <c r="R156" t="n">
         <v>66620</v>
-      </c>
-      <c r="R156" t="n">
-        <v>0</v>
       </c>
       <c r="S156" t="inlineStr"/>
       <c r="T156" t="inlineStr"/>
@@ -11068,10 +11068,10 @@
         </is>
       </c>
       <c r="Q157" t="n">
+        <v>0</v>
+      </c>
+      <c r="R157" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R157" t="n">
-        <v>0</v>
       </c>
       <c r="S157" t="inlineStr"/>
       <c r="T157" t="inlineStr"/>
@@ -11134,10 +11134,10 @@
         </is>
       </c>
       <c r="Q158" t="n">
+        <v>0</v>
+      </c>
+      <c r="R158" t="n">
         <v>2940000</v>
-      </c>
-      <c r="R158" t="n">
-        <v>0</v>
       </c>
       <c r="S158" t="inlineStr"/>
       <c r="T158" t="inlineStr"/>
@@ -11200,10 +11200,10 @@
         </is>
       </c>
       <c r="Q159" t="n">
+        <v>0</v>
+      </c>
+      <c r="R159" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R159" t="n">
-        <v>0</v>
       </c>
       <c r="S159" t="inlineStr"/>
       <c r="T159" t="inlineStr"/>
@@ -11266,10 +11266,10 @@
         </is>
       </c>
       <c r="Q160" t="n">
+        <v>0</v>
+      </c>
+      <c r="R160" t="n">
         <v>542000</v>
-      </c>
-      <c r="R160" t="n">
-        <v>0</v>
       </c>
       <c r="S160" t="inlineStr"/>
       <c r="T160" t="inlineStr"/>
@@ -11332,10 +11332,10 @@
         </is>
       </c>
       <c r="Q161" t="n">
+        <v>0</v>
+      </c>
+      <c r="R161" t="n">
         <v>2163814</v>
-      </c>
-      <c r="R161" t="n">
-        <v>0</v>
       </c>
       <c r="S161" t="inlineStr"/>
       <c r="T161" t="inlineStr"/>
@@ -11398,10 +11398,10 @@
         </is>
       </c>
       <c r="Q162" t="n">
+        <v>0</v>
+      </c>
+      <c r="R162" t="n">
         <v>11974837</v>
-      </c>
-      <c r="R162" t="n">
-        <v>0</v>
       </c>
       <c r="S162" t="inlineStr"/>
       <c r="T162" t="inlineStr"/>
@@ -11464,10 +11464,10 @@
         </is>
       </c>
       <c r="Q163" t="n">
+        <v>0</v>
+      </c>
+      <c r="R163" t="n">
         <v>1382535</v>
-      </c>
-      <c r="R163" t="n">
-        <v>0</v>
       </c>
       <c r="S163" t="inlineStr"/>
       <c r="T163" t="inlineStr"/>
@@ -11530,10 +11530,10 @@
         </is>
       </c>
       <c r="Q164" t="n">
+        <v>0</v>
+      </c>
+      <c r="R164" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R164" t="n">
-        <v>0</v>
       </c>
       <c r="S164" t="inlineStr"/>
       <c r="T164" t="inlineStr"/>
@@ -11596,10 +11596,10 @@
         </is>
       </c>
       <c r="Q165" t="n">
+        <v>0</v>
+      </c>
+      <c r="R165" t="n">
         <v>35359853</v>
-      </c>
-      <c r="R165" t="n">
-        <v>0</v>
       </c>
       <c r="S165" t="inlineStr"/>
       <c r="T165" t="inlineStr"/>
@@ -11662,10 +11662,10 @@
         </is>
       </c>
       <c r="Q166" t="n">
+        <v>0</v>
+      </c>
+      <c r="R166" t="n">
         <v>13982612</v>
-      </c>
-      <c r="R166" t="n">
-        <v>0</v>
       </c>
       <c r="S166" t="inlineStr"/>
       <c r="T166" t="inlineStr"/>
@@ -11728,10 +11728,10 @@
         </is>
       </c>
       <c r="Q167" t="n">
+        <v>0</v>
+      </c>
+      <c r="R167" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R167" t="n">
-        <v>0</v>
       </c>
       <c r="S167" t="inlineStr"/>
       <c r="T167" t="inlineStr"/>
@@ -11794,10 +11794,10 @@
         </is>
       </c>
       <c r="Q168" t="n">
+        <v>0</v>
+      </c>
+      <c r="R168" t="n">
         <v>10459632</v>
-      </c>
-      <c r="R168" t="n">
-        <v>0</v>
       </c>
       <c r="S168" t="inlineStr"/>
       <c r="T168" t="inlineStr"/>
@@ -11860,10 +11860,10 @@
         </is>
       </c>
       <c r="Q169" t="n">
+        <v>0</v>
+      </c>
+      <c r="R169" t="n">
         <v>17000000</v>
-      </c>
-      <c r="R169" t="n">
-        <v>0</v>
       </c>
       <c r="S169" t="inlineStr"/>
       <c r="T169" t="inlineStr"/>
@@ -11926,10 +11926,10 @@
         </is>
       </c>
       <c r="Q170" t="n">
+        <v>0</v>
+      </c>
+      <c r="R170" t="n">
         <v>74941121</v>
-      </c>
-      <c r="R170" t="n">
-        <v>0</v>
       </c>
       <c r="S170" t="inlineStr"/>
       <c r="T170" t="inlineStr"/>
@@ -11992,10 +11992,10 @@
         </is>
       </c>
       <c r="Q171" t="n">
+        <v>0</v>
+      </c>
+      <c r="R171" t="n">
         <v>38460000</v>
-      </c>
-      <c r="R171" t="n">
-        <v>0</v>
       </c>
       <c r="S171" t="inlineStr"/>
       <c r="T171" t="inlineStr"/>
@@ -12058,10 +12058,10 @@
         </is>
       </c>
       <c r="Q172" t="n">
+        <v>0</v>
+      </c>
+      <c r="R172" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R172" t="n">
-        <v>0</v>
       </c>
       <c r="S172" t="inlineStr"/>
       <c r="T172" t="inlineStr"/>
@@ -12124,10 +12124,10 @@
         </is>
       </c>
       <c r="Q173" t="n">
+        <v>0</v>
+      </c>
+      <c r="R173" t="n">
         <v>7000000</v>
-      </c>
-      <c r="R173" t="n">
-        <v>0</v>
       </c>
       <c r="S173" t="inlineStr"/>
       <c r="T173" t="inlineStr"/>
@@ -12190,10 +12190,10 @@
         </is>
       </c>
       <c r="Q174" t="n">
+        <v>0</v>
+      </c>
+      <c r="R174" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R174" t="n">
-        <v>0</v>
       </c>
       <c r="S174" t="inlineStr"/>
       <c r="T174" t="inlineStr"/>
@@ -12784,10 +12784,10 @@
         </is>
       </c>
       <c r="Q183" t="n">
+        <v>0</v>
+      </c>
+      <c r="R183" t="n">
         <v>100000</v>
-      </c>
-      <c r="R183" t="n">
-        <v>0</v>
       </c>
       <c r="S183" t="inlineStr"/>
       <c r="T183" t="inlineStr"/>
@@ -12850,10 +12850,10 @@
         </is>
       </c>
       <c r="Q184" t="n">
+        <v>0</v>
+      </c>
+      <c r="R184" t="n">
         <v>6121132</v>
-      </c>
-      <c r="R184" t="n">
-        <v>0</v>
       </c>
       <c r="S184" t="inlineStr"/>
       <c r="T184" t="inlineStr"/>
@@ -12916,10 +12916,10 @@
         </is>
       </c>
       <c r="Q185" t="n">
+        <v>0</v>
+      </c>
+      <c r="R185" t="n">
         <v>3541728</v>
-      </c>
-      <c r="R185" t="n">
-        <v>0</v>
       </c>
       <c r="S185" t="inlineStr"/>
       <c r="T185" t="inlineStr"/>
@@ -12982,10 +12982,10 @@
         </is>
       </c>
       <c r="Q186" t="n">
+        <v>0</v>
+      </c>
+      <c r="R186" t="n">
         <v>22254062</v>
-      </c>
-      <c r="R186" t="n">
-        <v>0</v>
       </c>
       <c r="S186" t="inlineStr"/>
       <c r="T186" t="inlineStr"/>
@@ -13048,10 +13048,10 @@
         </is>
       </c>
       <c r="Q187" t="n">
+        <v>0</v>
+      </c>
+      <c r="R187" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R187" t="n">
-        <v>0</v>
       </c>
       <c r="S187" t="inlineStr"/>
       <c r="T187" t="inlineStr"/>
@@ -13114,10 +13114,10 @@
         </is>
       </c>
       <c r="Q188" t="n">
+        <v>0</v>
+      </c>
+      <c r="R188" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R188" t="n">
-        <v>0</v>
       </c>
       <c r="S188" t="inlineStr"/>
       <c r="T188" t="inlineStr"/>
@@ -13180,10 +13180,10 @@
         </is>
       </c>
       <c r="Q189" t="n">
+        <v>0</v>
+      </c>
+      <c r="R189" t="n">
         <v>431809</v>
-      </c>
-      <c r="R189" t="n">
-        <v>0</v>
       </c>
       <c r="S189" t="inlineStr"/>
       <c r="T189" t="inlineStr"/>
@@ -13246,10 +13246,10 @@
         </is>
       </c>
       <c r="Q190" t="n">
+        <v>0</v>
+      </c>
+      <c r="R190" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R190" t="n">
-        <v>0</v>
       </c>
       <c r="S190" t="inlineStr"/>
       <c r="T190" t="inlineStr"/>
@@ -13312,10 +13312,10 @@
         </is>
       </c>
       <c r="Q191" t="n">
+        <v>0</v>
+      </c>
+      <c r="R191" t="n">
         <v>14356790</v>
-      </c>
-      <c r="R191" t="n">
-        <v>0</v>
       </c>
       <c r="S191" t="inlineStr"/>
       <c r="T191" t="inlineStr"/>
@@ -13378,10 +13378,10 @@
         </is>
       </c>
       <c r="Q192" t="n">
+        <v>0</v>
+      </c>
+      <c r="R192" t="n">
         <v>1000</v>
-      </c>
-      <c r="R192" t="n">
-        <v>0</v>
       </c>
       <c r="S192" t="inlineStr"/>
       <c r="T192" t="inlineStr"/>
@@ -13444,10 +13444,10 @@
         </is>
       </c>
       <c r="Q193" t="n">
+        <v>0</v>
+      </c>
+      <c r="R193" t="n">
         <v>1000</v>
-      </c>
-      <c r="R193" t="n">
-        <v>0</v>
       </c>
       <c r="S193" t="inlineStr"/>
       <c r="T193" t="inlineStr"/>
@@ -13972,10 +13972,10 @@
         </is>
       </c>
       <c r="Q201" t="n">
+        <v>0</v>
+      </c>
+      <c r="R201" t="n">
         <v>50000000</v>
-      </c>
-      <c r="R201" t="n">
-        <v>0</v>
       </c>
       <c r="S201" t="inlineStr"/>
       <c r="T201" t="inlineStr"/>
@@ -14038,10 +14038,10 @@
         </is>
       </c>
       <c r="Q202" t="n">
+        <v>0</v>
+      </c>
+      <c r="R202" t="n">
         <v>8151612</v>
-      </c>
-      <c r="R202" t="n">
-        <v>0</v>
       </c>
       <c r="S202" t="inlineStr"/>
       <c r="T202" t="inlineStr"/>
@@ -14104,10 +14104,10 @@
         </is>
       </c>
       <c r="Q203" t="n">
+        <v>0</v>
+      </c>
+      <c r="R203" t="n">
         <v>7488179</v>
-      </c>
-      <c r="R203" t="n">
-        <v>0</v>
       </c>
       <c r="S203" t="inlineStr"/>
       <c r="T203" t="inlineStr"/>
@@ -14170,10 +14170,10 @@
         </is>
       </c>
       <c r="Q204" t="n">
+        <v>0</v>
+      </c>
+      <c r="R204" t="n">
         <v>9608804</v>
-      </c>
-      <c r="R204" t="n">
-        <v>0</v>
       </c>
       <c r="S204" t="inlineStr"/>
       <c r="T204" t="inlineStr"/>
@@ -14236,10 +14236,10 @@
         </is>
       </c>
       <c r="Q205" t="n">
+        <v>0</v>
+      </c>
+      <c r="R205" t="n">
         <v>8168067</v>
-      </c>
-      <c r="R205" t="n">
-        <v>0</v>
       </c>
       <c r="S205" t="inlineStr"/>
       <c r="T205" t="inlineStr"/>
@@ -14302,10 +14302,10 @@
         </is>
       </c>
       <c r="Q206" t="n">
+        <v>0</v>
+      </c>
+      <c r="R206" t="n">
         <v>571386707</v>
-      </c>
-      <c r="R206" t="n">
-        <v>0</v>
       </c>
       <c r="S206" t="inlineStr"/>
       <c r="T206" t="inlineStr"/>
@@ -14368,10 +14368,10 @@
         </is>
       </c>
       <c r="Q207" t="n">
+        <v>0</v>
+      </c>
+      <c r="R207" t="n">
         <v>15000000</v>
-      </c>
-      <c r="R207" t="n">
-        <v>0</v>
       </c>
       <c r="S207" t="inlineStr"/>
       <c r="T207" t="inlineStr"/>
@@ -14434,10 +14434,10 @@
         </is>
       </c>
       <c r="Q208" t="n">
+        <v>0</v>
+      </c>
+      <c r="R208" t="n">
         <v>1406178</v>
-      </c>
-      <c r="R208" t="n">
-        <v>0</v>
       </c>
       <c r="S208" t="inlineStr"/>
       <c r="T208" t="inlineStr"/>
@@ -14500,10 +14500,10 @@
         </is>
       </c>
       <c r="Q209" t="n">
+        <v>0</v>
+      </c>
+      <c r="R209" t="n">
         <v>19448656</v>
-      </c>
-      <c r="R209" t="n">
-        <v>0</v>
       </c>
       <c r="S209" t="inlineStr"/>
       <c r="T209" t="inlineStr"/>
@@ -14566,10 +14566,10 @@
         </is>
       </c>
       <c r="Q210" t="n">
+        <v>0</v>
+      </c>
+      <c r="R210" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R210" t="n">
-        <v>0</v>
       </c>
       <c r="S210" t="inlineStr"/>
       <c r="T210" t="inlineStr"/>
@@ -14632,10 +14632,10 @@
         </is>
       </c>
       <c r="Q211" t="n">
+        <v>0</v>
+      </c>
+      <c r="R211" t="n">
         <v>30000000</v>
-      </c>
-      <c r="R211" t="n">
-        <v>0</v>
       </c>
       <c r="S211" t="inlineStr"/>
       <c r="T211" t="inlineStr"/>
@@ -14698,10 +14698,10 @@
         </is>
       </c>
       <c r="Q212" t="n">
+        <v>0</v>
+      </c>
+      <c r="R212" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R212" t="n">
-        <v>0</v>
       </c>
       <c r="S212" t="inlineStr"/>
       <c r="T212" t="inlineStr"/>
@@ -14764,10 +14764,10 @@
         </is>
       </c>
       <c r="Q213" t="n">
+        <v>0</v>
+      </c>
+      <c r="R213" t="n">
         <v>4000000</v>
-      </c>
-      <c r="R213" t="n">
-        <v>0</v>
       </c>
       <c r="S213" t="inlineStr"/>
       <c r="T213" t="inlineStr"/>
@@ -14830,10 +14830,10 @@
         </is>
       </c>
       <c r="Q214" t="n">
+        <v>0</v>
+      </c>
+      <c r="R214" t="n">
         <v>4000000</v>
-      </c>
-      <c r="R214" t="n">
-        <v>0</v>
       </c>
       <c r="S214" t="inlineStr"/>
       <c r="T214" t="inlineStr"/>
@@ -14896,10 +14896,10 @@
         </is>
       </c>
       <c r="Q215" t="n">
+        <v>0</v>
+      </c>
+      <c r="R215" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R215" t="n">
-        <v>0</v>
       </c>
       <c r="S215" t="inlineStr"/>
       <c r="T215" t="inlineStr"/>
@@ -15300,10 +15300,10 @@
         </is>
       </c>
       <c r="Q221" t="n">
+        <v>0</v>
+      </c>
+      <c r="R221" t="n">
         <v>8311374</v>
-      </c>
-      <c r="R221" t="n">
-        <v>0</v>
       </c>
       <c r="S221" t="inlineStr"/>
       <c r="T221" t="inlineStr"/>
@@ -15366,10 +15366,10 @@
         </is>
       </c>
       <c r="Q222" t="n">
+        <v>0</v>
+      </c>
+      <c r="R222" t="n">
         <v>477508</v>
-      </c>
-      <c r="R222" t="n">
-        <v>0</v>
       </c>
       <c r="S222" t="inlineStr"/>
       <c r="T222" t="inlineStr"/>

</xml_diff>